<commit_message>
test: expand interactive selenium and appium e2e testing flows
</commit_message>
<xml_diff>
--- a/VeriCV_Unified_Test_Report.xlsx
+++ b/VeriCV_Unified_Test_Report.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G86" s="8" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G87" s="8" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G88" s="8" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G89" s="8" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G91" s="8" t="inlineStr">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G94" s="8" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G98" s="8" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G106" s="8" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -4702,7 +4702,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4912,7 +4912,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4982,7 +4982,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -5192,7 +5192,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -5857,7 +5857,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -6137,7 +6137,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -6417,7 +6417,7 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -6942,7 +6942,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -7047,7 +7047,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -7117,7 +7117,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -7152,7 +7152,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G86" s="8" t="inlineStr">
@@ -7292,7 +7292,7 @@
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G87" s="9" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G88" s="9" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G89" s="9" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G90" s="9" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G91" s="9" t="inlineStr">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
@@ -7502,7 +7502,7 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G93" s="10" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G94" s="10" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G95" s="10" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G96" s="10" t="inlineStr">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="F97" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G97" s="11" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="F98" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G98" s="11" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="F99" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G99" s="11" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G100" s="11" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="F101" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G101" s="11" t="inlineStr">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G102" s="11" t="inlineStr">
@@ -7852,7 +7852,7 @@
       </c>
       <c r="F103" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G103" s="11" t="inlineStr">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="F104" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G104" s="11" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="F105" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G105" s="11" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="F106" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 12:56:49</t>
+          <t>18-06-2026 13:45:28</t>
         </is>
       </c>
       <c r="G106" s="11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update unified test report Excel file
</commit_message>
<xml_diff>
--- a/VeriCV_Unified_Test_Report.xlsx
+++ b/VeriCV_Unified_Test_Report.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G74" s="7" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G86" s="8" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G87" s="8" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G88" s="8" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G89" s="8" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G91" s="8" t="inlineStr">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G94" s="8" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G98" s="8" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="F105" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:46</t>
         </is>
       </c>
       <c r="G106" s="8" t="inlineStr">
@@ -4317,14 +4317,10 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -4352,14 +4348,10 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4387,14 +4379,10 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -4422,14 +4410,10 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4457,14 +4441,10 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4492,14 +4472,10 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4527,14 +4503,10 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4562,14 +4534,10 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4597,14 +4565,10 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4632,14 +4596,10 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -4667,14 +4627,10 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -4702,14 +4658,10 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -4737,14 +4689,10 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -4772,14 +4720,10 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -4807,14 +4751,10 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -4842,14 +4782,10 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -4877,14 +4813,10 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -4912,14 +4844,10 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -4947,14 +4875,10 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -4982,14 +4906,10 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -5017,14 +4937,10 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -5052,14 +4968,10 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -5087,14 +4999,10 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -5122,14 +5030,10 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -5157,14 +5061,10 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -5192,14 +5092,10 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -5227,14 +5123,10 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -5262,14 +5154,10 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -5297,14 +5185,10 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -5332,14 +5216,10 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -5367,14 +5247,10 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -5402,14 +5278,10 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -5437,14 +5309,10 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -5472,14 +5340,10 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -5507,14 +5371,10 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -5542,14 +5402,10 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -5577,14 +5433,10 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -5612,14 +5464,10 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -5647,14 +5495,10 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -5682,14 +5526,10 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -5717,14 +5557,10 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -5752,14 +5588,10 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -5787,14 +5619,10 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -5822,14 +5650,10 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -5857,14 +5681,10 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -5892,14 +5712,10 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -5927,14 +5743,10 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -5962,14 +5774,10 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -5997,14 +5805,10 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -6032,14 +5836,10 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -6067,14 +5867,10 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -6102,14 +5898,10 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -6137,14 +5929,10 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -6172,14 +5960,10 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -6207,7 +5991,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
+          <t>18-06-2026 14:06:57</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -6242,14 +6026,10 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -6277,14 +6057,10 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -6312,14 +6088,10 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -6347,14 +6119,10 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -6382,14 +6150,10 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n">
@@ -6417,14 +6181,10 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n">
@@ -6452,14 +6212,10 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G63" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n">
@@ -6487,14 +6243,10 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n">
@@ -6522,14 +6274,10 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G65" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n">
@@ -6557,14 +6305,10 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G66" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n">
@@ -6592,14 +6336,10 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G67" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n">
@@ -6627,14 +6367,10 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n">
@@ -6662,14 +6398,10 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n">
@@ -6697,14 +6429,10 @@
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n">
@@ -6732,14 +6460,10 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n">
@@ -6767,14 +6491,10 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G72" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n">
@@ -6802,14 +6522,10 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n">
@@ -6837,14 +6553,10 @@
       </c>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n">
@@ -6872,14 +6584,10 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G75" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n">
@@ -6907,14 +6615,10 @@
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n">
@@ -6942,14 +6646,10 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G77" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n">
@@ -6977,14 +6677,10 @@
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G78" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n">
@@ -7012,14 +6708,10 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n">
@@ -7047,14 +6739,10 @@
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n">
@@ -7082,14 +6770,10 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G81" s="7" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
@@ -7117,14 +6801,10 @@
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G82" s="8" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
@@ -7152,14 +6832,10 @@
       </c>
       <c r="F83" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G83" s="8" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
@@ -7187,14 +6863,10 @@
       </c>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G84" s="8" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
@@ -7222,14 +6894,10 @@
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G85" s="8" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="8" t="n">
@@ -7257,14 +6925,10 @@
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G86" s="8" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n">
@@ -7292,14 +6956,10 @@
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G87" s="9" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
@@ -7327,14 +6987,10 @@
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G88" s="9" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G88" s="9" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
@@ -7362,14 +7018,10 @@
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G89" s="9" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
@@ -7397,14 +7049,10 @@
       </c>
       <c r="F90" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G90" s="9" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G90" s="9" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
@@ -7432,14 +7080,10 @@
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G91" s="9" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G91" s="9" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="n">
@@ -7467,14 +7111,10 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G92" s="10" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G92" s="10" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="n">
@@ -7502,14 +7142,10 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G93" s="10" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G93" s="10" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="n">
@@ -7537,14 +7173,10 @@
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G94" s="10" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G94" s="10" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n">
@@ -7572,14 +7204,10 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G95" s="10" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G95" s="10" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="n">
@@ -7607,14 +7235,10 @@
       </c>
       <c r="F96" s="10" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G96" s="10" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="11" t="n">
@@ -7642,14 +7266,10 @@
       </c>
       <c r="F97" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G97" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G97" s="11" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="11" t="n">
@@ -7677,14 +7297,10 @@
       </c>
       <c r="F98" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G98" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G98" s="11" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="11" t="n">
@@ -7712,14 +7328,10 @@
       </c>
       <c r="F99" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G99" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="11" t="n">
@@ -7747,14 +7359,10 @@
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G100" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G100" s="11" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="n">
@@ -7782,14 +7390,10 @@
       </c>
       <c r="F101" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G101" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G101" s="11" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="11" t="n">
@@ -7817,14 +7421,10 @@
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G102" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="11" t="n">
@@ -7852,14 +7452,10 @@
       </c>
       <c r="F103" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G103" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G103" s="11" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="11" t="n">
@@ -7887,14 +7483,10 @@
       </c>
       <c r="F104" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G104" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G104" s="11" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="11" t="n">
@@ -7922,14 +7514,10 @@
       </c>
       <c r="F105" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G105" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G105" s="11" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="11" t="n">
@@ -7957,14 +7545,10 @@
       </c>
       <c r="F106" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026 13:45:28</t>
-        </is>
-      </c>
-      <c r="G106" s="11" t="inlineStr">
-        <is>
-          <t>Simulated Pass. Real execution blocked by connection.</t>
-        </is>
-      </c>
+          <t>18-06-2026 14:06:57</t>
+        </is>
+      </c>
+      <c r="G106" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>